<commit_message>
feat(numerical): land aug-sep production batch with final docs and chg audits
- 数值生产：收录 04_数值文档 终稿、05_验算核算（CHG010-012、CHG019-026、难度重算、SVN 落表差异）与 06_最终配置 镜像
- 沉淀与知识：03_沉淀MD 增量、knowledge-base 数值域与经验条目、知识图谱重建
- 设计文档：战力系统、映射装备数值爆改与占位彩装屏蔽、房车等级挂钩、资源副本五层重构等
- 工程卫生：22 个脚本与文档的硬编码盘符路径改为 vgame_paths/环境变量解析（本机解析值不变）；.gitignore 增加 tmp/ 与本地工具目录
</commit_message>
<xml_diff>
--- a/numerical-workflows/v2/framework/01_源表/节奏口径.xlsx
+++ b/numerical-workflows/v2/framework/01_源表/节奏口径.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\数值文档\数值文档\框架v2\01_源表\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vgame_design\numerical-workflows\v2\framework\01_源表\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -117,7 +117,7 @@
     <t>舱室</t>
   </si>
   <si>
-    <t>资源副本-舱室</t>
+    <t>资源副本-舱室、温泉</t>
   </si>
   <si>
     <t>舱室养成需要建筑材料，可以从主线和高难主线刷取</t>

</xml_diff>